<commit_message>
feat: initialize research workspace with literature review matrix and edge sleep staging blueprint
</commit_message>
<xml_diff>
--- a/Literature_Review_Matrix.xlsx
+++ b/Literature_Review_Matrix.xlsx
@@ -454,7 +454,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -600,6 +600,15 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="16" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1441,7 +1450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH25"/>
+  <dimension ref="A1:BH26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2045,12 +2054,12 @@
     <row r="5" ht="54.75" customHeight="1">
       <c r="A5" s="25" t="inlineStr">
         <is>
-          <t>P002</t>
+          <t>P001</t>
         </is>
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>Phan et al. (2019). SeqSleepNet: End-to-End Hierarchical Recurrent Neural Network for Sequence-to-Sequence Automatic Sleep Staging.</t>
+          <t>DeepSleepNet: a Model for Automatic Sleep Stage Scoring based on Raw Single-Channel EEG Akara Supratak, Hao Dong, Chao Wu, and Yike Guo*</t>
         </is>
       </c>
       <c r="C5" s="25" t="inlineStr">
@@ -2345,12 +2354,12 @@
     <row r="6" ht="50.25" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>P003</t>
+          <t>P002</t>
         </is>
       </c>
       <c r="B6" s="24" t="inlineStr">
         <is>
-          <t>Li &amp; Gao (2023). Automatic sleep staging by a hybrid model based on deep 1D-ResNet-SE and LSTM with single-channel raw EEG signals.</t>
+          <t>arXiv:1809.10932v3  [cs.LG]  2 Feb 2019 SeqSleepNet: End-to-End Hierarchical Recurrent Neural Network for Sequence-to-Sequence</t>
         </is>
       </c>
       <c r="C6" s="24" t="inlineStr">
@@ -2645,12 +2654,12 @@
     <row r="7" ht="50.25" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>P004</t>
+          <t>P003</t>
         </is>
       </c>
       <c r="B7" s="25" t="inlineStr">
         <is>
-          <t>Eldele et al. (2021). An Attention-Based Deep Learning Approach for Sleep Stage Classification With Single-Channel EEG.</t>
+          <t>Article 1 Automatic sleep staging by a hybrid model based on deep 1D- 2 ResNet-SE and LSTM with single-channel raw EEG signals 3</t>
         </is>
       </c>
       <c r="C7" s="25" t="inlineStr">
@@ -2945,12 +2954,12 @@
     <row r="8" ht="50.25" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>P005</t>
+          <t>P004</t>
         </is>
       </c>
       <c r="B8" s="24" t="inlineStr">
         <is>
-          <t>Author(s) (Year). An Unsupervised TinyML Approach with Efficient Edge AI for Effective Stress and Sleep Monitoring.</t>
+          <t>An Attention-Based Deep Learning Approach for Sleep Stage Classiﬁcation With Single-Channel EEG</t>
         </is>
       </c>
       <c r="C8" s="24" t="inlineStr">
@@ -3245,12 +3254,12 @@
     <row r="9" ht="50.25" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
         <is>
-          <t>P006</t>
+          <t>P005</t>
         </is>
       </c>
       <c r="B9" s="25" t="inlineStr">
         <is>
-          <t>Author(s) (Year). A Smart System for Sleep Monitoring by Integrating IoT With Big Data Analytics.</t>
+          <t>1 An Unsupervised TinyML Approach with Efficient Edge AI for Effective Stress and Sleep</t>
         </is>
       </c>
       <c r="C9" s="25" t="inlineStr">
@@ -3545,12 +3554,12 @@
     <row r="10" ht="50.25" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>P007</t>
+          <t>P006</t>
         </is>
       </c>
       <c r="B10" s="24" t="inlineStr">
         <is>
-          <t>Author(s) (Year). bioengineering-12-01191-v2.</t>
+          <t>Digital Object Identifier 10.1 109/ACCESS.2018.2849822 A Smart System for Sleep Monitoring by Integrating IoT With Big Data Analytics</t>
         </is>
       </c>
       <c r="C10" s="24" t="inlineStr">
@@ -3845,12 +3854,12 @@
     <row r="11" ht="50.25" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>P008</t>
+          <t>P007</t>
         </is>
       </c>
       <c r="B11" s="25" t="inlineStr">
         <is>
-          <t>Author(s) (Year). engproc-78-00003-v2.</t>
+          <t>Academic Editor: Luca Mesin Revised: 28 October 2025 Published: 31 October 2025</t>
         </is>
       </c>
       <c r="C11" s="25" t="inlineStr">
@@ -4145,12 +4154,12 @@
     <row r="12" ht="50.25" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>P009</t>
+          <t>P008</t>
         </is>
       </c>
       <c r="B12" s="24" t="inlineStr">
         <is>
-          <t>Author(s) (Year). Federated-Learning-for-Sleep-Stage-Classification-on-Edge-Devices-via-a-Model-Agnostic-Meta.</t>
+          <t>Citation: Srivastava, P .; Shah, N.; Jaiswal, K. Microcontroller-Based EdgeML: Health Monitoring for Stress</t>
         </is>
       </c>
       <c r="C12" s="24" t="inlineStr">
@@ -4445,12 +4454,12 @@
     <row r="13" ht="50.25" customHeight="1">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>P010</t>
+          <t>P009</t>
         </is>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>Author(s) (Year). j.1365-2869.2011.00944.x.</t>
+          <t>Federated Learning for Sleep Stage Classification on Edge Devices via a Model-Agnostic Meta-Learning-Based Pre-Trained Model</t>
         </is>
       </c>
       <c r="C13" s="25" t="inlineStr">
@@ -4745,12 +4754,12 @@
     <row r="14" ht="50.25" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P011</t>
+          <t>P010</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Author(s) (Year). jmir-2025-1-e65272.</t>
+          <t>Validation of an automated wireless system to monitor sleep in healthy adults JOHN R. SHAMBROOM 1 , STEPHAN E. FA ´ BREGAS 1 and JACK JOHNSTONE 2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -5045,12 +5054,12 @@
     <row r="15" ht="50.25" customHeight="1">
       <c r="A15" t="inlineStr">
         <is>
-          <t>P012</t>
+          <t>P011</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Liu et al. (2022). Multi-scale ResNet and BiGRU automatic sleep staging based on attention mechanism. PLOS ONE 17(6): e0269500.</t>
+          <t>Review Wearable Artificial Intelligence for Sleep Disorders: Scoping Review</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -5345,12 +5354,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>P013</t>
+          <t>P012</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Author(s) (Year). journal.pone.0285703.</t>
+          <t>RESEA RCH ARTICL E Multi-scale ResNet and BiGRU automatic sleep staging based on attention mechanism</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -5645,12 +5654,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>P014</t>
+          <t>P013</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Author(s) (Year). journal.pone.0332577.</t>
+          <t>RESEA RCH ARTICL E AI-Driven sleep staging from actigraphy and heart rate</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5945,12 +5954,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>P015</t>
+          <t>P014</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Author(s) (Year). PDF.pdf</t>
+          <t>ID: pone.0332577 — 2025/11/1 — page 1 — #1 PLOS ONE OPEN ACCESS</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -6245,12 +6254,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P016</t>
+          <t>P015</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Author(s) (Year). s41746-024-01086-9.</t>
+          <t>Review Detection of Sleep Apnea Using Wearable AI: Systematic Review and Meta-Analysis</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -6545,12 +6554,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>P017</t>
+          <t>P016</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Author(s) (Year). sensors-23-04950.</t>
+          <t>npj |digital medicine Editorial Published in partnership with Seoul National University Bundang Hospital Challenges and opportunities of deep learning</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -6845,12 +6854,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>P018</t>
+          <t>P017</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Author(s) (Year). sensors-23-05696-v2.</t>
+          <t>Citation: Toma, T.I.; Choi, S. An End-to-End Multi-Channel Convolutional Bi-LSTM Network for</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -7145,12 +7154,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>P019</t>
+          <t>P018</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Author(s) (Year). sensors-26-01803-v2.</t>
+          <t>Citation: Alajlan, N.N.; Ibrahim, D.M. DDD TinyML: A TinyML-Based Driver Drowsiness Detection Model</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -7445,12 +7454,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>P020</t>
+          <t>P019</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Author(s) (Year). SleepFCN: A Fully Convolutional Deep Learning Framework for Sleep Stage Classification Using Single-Channel Electroencephalograms.</t>
+          <t>Academic Editor: Miguel Ángel Carvajal Rodríguez Revised: 3 March 2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -7745,12 +7754,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>P021</t>
+          <t>P020</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Zhu et al. (2021). zhu2021.</t>
+          <t>SleepFCN: A Fully Convolutional Deep Learning Framework for Sleep Stage Classiﬁcation Using Single-Channel Electroencephalograms</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -8045,12 +8054,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P022</t>
+          <t>P021</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Author(s) (Year). zsae187.</t>
+          <t>Vol.:(0123456789) 1 3 A lightweight automatic sleep staging method for children</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -8339,6 +8348,18 @@
       <c r="BH25" t="inlineStr">
         <is>
           <t>Generic zsae187 paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>P022</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SLEEP, 2025, 48, 1–14 Advance access publication 19 August 2024 Original Article</t>
         </is>
       </c>
     </row>
@@ -8394,7 +8415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8502,12 +8523,12 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
         <is>
-          <t>G001</t>
+          <t>P001</t>
         </is>
       </c>
       <c r="B4" s="24" t="inlineStr">
         <is>
-          <t>No cross-subject transfer learning evaluated for EEG motor imagery BCI systems in real-world noisy conditions</t>
+          <t>DeepSleepNet: a Model for Automatic Sleep Stage Scoring based on Raw Single-Channel EEG Akara Supratak, Hao Dong, Chao Wu, and Yike Guo*</t>
         </is>
       </c>
       <c r="C4" s="24" t="inlineStr">
@@ -8515,9 +8536,9 @@
           <t>P001, P004</t>
         </is>
       </c>
-      <c r="D4" s="24" t="inlineStr">
-        <is>
-          <t>Neuroscience / ML</t>
+      <c r="D4" s="54" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
         </is>
       </c>
       <c r="E4" s="24" t="inlineStr">
@@ -8567,12 +8588,12 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="25" t="inlineStr">
         <is>
-          <t>G002</t>
+          <t>P002</t>
         </is>
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>FPGA-based real-time inference for bio-signal data (EEG/ECG) remains unexplored vs. image-only FPGA acceleration</t>
+          <t>arXiv:1809.10932v3  [cs.LG]  2 Feb 2019 SeqSleepNet: End-to-End Hierarchical Recurrent Neural Network for Sequence-to-Sequence</t>
         </is>
       </c>
       <c r="C5" s="25" t="inlineStr">
@@ -8580,9 +8601,9 @@
           <t>P003, P005</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
-        <is>
-          <t>Electronics / Embedded AI</t>
+      <c r="D5" s="55" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
         </is>
       </c>
       <c r="E5" s="25" t="inlineStr">
@@ -8632,17 +8653,21 @@
     <row r="6" ht="50.25" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>G003</t>
-        </is>
-      </c>
-      <c r="B6" s="24" t="n">
-        <v>0</v>
+          <t>P003</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Article 1 Automatic sleep staging by a hybrid model based on deep 1D- 2 ResNet-SE and LSTM with single-channel raw EEG signals 3</t>
+        </is>
       </c>
       <c r="C6" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="24" t="n">
-        <v>0</v>
+      <c r="D6" s="54" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
       </c>
       <c r="E6" s="24" t="n">
         <v>0</v>
@@ -8678,17 +8703,21 @@
     <row r="7" ht="50.25" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>G004</t>
-        </is>
-      </c>
-      <c r="B7" s="25" t="n">
-        <v>0</v>
+          <t>P004</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>An Attention-Based Deep Learning Approach for Sleep Stage Classiﬁcation With Single-Channel EEG</t>
+        </is>
       </c>
       <c r="C7" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="25" t="n">
-        <v>0</v>
+      <c r="D7" s="55" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
       </c>
       <c r="E7" s="25" t="n">
         <v>0</v>
@@ -8724,17 +8753,21 @@
     <row r="8" ht="50.25" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>G005</t>
-        </is>
-      </c>
-      <c r="B8" s="24" t="n">
-        <v>0</v>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>1 An Unsupervised TinyML Approach with Efficient Edge AI for Effective Stress and Sleep</t>
+        </is>
       </c>
       <c r="C8" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="24" t="n">
-        <v>0</v>
+      <c r="D8" s="54" t="inlineStr">
+        <is>
+          <t>The proposed UTMESS is mainly designed to  monitor the physiological states in real time through  the presence of edge computing, multi-sensor fusion,  and deep learning. It uses I MU and HRV data from  ISRUC and SWELL datasets, to improve the feature  extraction. The proposed UTMESS has a dual  architecture featuring a MobileNetV2 classifier for  sleep and stress detection and an LSTM autoencoder  for finding abnormalities. It handles bo th sequential  and static signals in an effective man...</t>
+        </is>
       </c>
       <c r="E8" s="24" t="n">
         <v>0</v>
@@ -8770,17 +8803,21 @@
     <row r="9" ht="50.25" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
         <is>
-          <t>G006</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="n">
-        <v>0</v>
+          <t>P006</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>Digital Object Identifier 10.1 109/ACCESS.2018.2849822 A Smart System for Sleep Monitoring by Integrating IoT With Big Data Analytics</t>
+        </is>
       </c>
       <c r="C9" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="25" t="n">
-        <v>0</v>
+      <c r="D9" s="55" t="inlineStr">
+        <is>
+          <t>in the future the number of older adults will represent more than 14% of the world’s population.</t>
+        </is>
       </c>
       <c r="E9" s="25" t="n">
         <v>0</v>
@@ -8816,17 +8853,21 @@
     <row r="10" ht="50.25" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>G007</t>
-        </is>
-      </c>
-      <c r="B10" s="24" t="n">
-        <v>0</v>
+          <t>P007</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>Academic Editor: Luca Mesin Revised: 28 October 2025 Published: 31 October 2025</t>
+        </is>
       </c>
       <c r="C10" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="24" t="n">
-        <v>0</v>
+      <c r="D10" s="54" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
       </c>
       <c r="E10" s="24" t="n">
         <v>0</v>
@@ -8862,17 +8903,21 @@
     <row r="11" ht="50.25" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>G008</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="n">
-        <v>0</v>
+          <t>P008</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>Citation: Srivastava, P .; Shah, N.; Jaiswal, K. Microcontroller-Based EdgeML: Health Monitoring for Stress</t>
+        </is>
       </c>
       <c r="C11" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="25" t="n">
-        <v>0</v>
+      <c r="D11" s="55" t="inlineStr">
+        <is>
+          <t>Future Work This paper demonstrates the successful deployment of a stress prediction model on a resource-constrained microcontroller, showing that advanced machine learning models can be effectively run on low-powered hardware without compromising accuracy.</t>
+        </is>
       </c>
       <c r="E11" s="25" t="n">
         <v>0</v>
@@ -8908,17 +8953,21 @@
     <row r="12" ht="50.25" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>G009</t>
-        </is>
-      </c>
-      <c r="B12" s="24" t="n">
-        <v>0</v>
+          <t>P009</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>Federated Learning for Sleep Stage Classification on Edge Devices via a Model-Agnostic Meta-Learning-Based Pre-Trained Model</t>
+        </is>
       </c>
       <c r="C12" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="24" t="n">
-        <v>0</v>
+      <c r="D12" s="54" t="inlineStr">
+        <is>
+          <t>AND CONCLUSIONS  In this study, we investigated the impact of initialization  strategies in FL for sleep stage classification, considering the  limited computational resources of edge devices. We  compared locally trained models, FL models with random  initialization, and FL models initialized with pre-trained  weights from the MAML model. Our findings demonstrated  that FL models, despite their decentralized training nature,  generally exhibited superior performance compared to locally  traine...</t>
+        </is>
       </c>
       <c r="E12" s="24" t="n">
         <v>0</v>
@@ -8954,17 +9003,21 @@
     <row r="13" ht="50.25" customHeight="1">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>G010</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="n">
-        <v>0</v>
+          <t>P010</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>Validation of an automated wireless system to monitor sleep in healthy adults JOHN R. SHAMBROOM 1 , STEPHAN E. FA ´ BREGAS 1 and JACK JOHNSTONE 2</t>
+        </is>
       </c>
       <c r="C13" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="25" t="n">
-        <v>0</v>
+      <c r="D13" s="55" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
       </c>
       <c r="E13" s="25" t="n">
         <v>0</v>
@@ -9000,17 +9053,21 @@
     <row r="14" ht="50.25" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>G011</t>
-        </is>
-      </c>
-      <c r="B14" s="24" t="n">
-        <v>0</v>
+          <t>P011</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>Review Wearable Artificial Intelligence for Sleep Disorders: Scoping Review</t>
+        </is>
       </c>
       <c r="C14" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="24" t="n">
-        <v>0</v>
+      <c r="D14" s="54" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
       </c>
       <c r="E14" s="24" t="n">
         <v>0</v>
@@ -9046,17 +9103,21 @@
     <row r="15" ht="50.25" customHeight="1">
       <c r="A15" s="25" t="inlineStr">
         <is>
-          <t>G012</t>
-        </is>
-      </c>
-      <c r="B15" s="25" t="n">
-        <v>0</v>
+          <t>P012</t>
+        </is>
+      </c>
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>RESEA RCH ARTICL E Multi-scale ResNet and BiGRU automatic sleep staging based on attention mechanism</t>
+        </is>
       </c>
       <c r="C15" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="25" t="n">
-        <v>0</v>
+      <c r="D15" s="55" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
       </c>
       <c r="E15" s="25" t="n">
         <v>0</v>
@@ -9092,17 +9153,21 @@
     <row r="16" ht="50.25" customHeight="1">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>G013</t>
-        </is>
-      </c>
-      <c r="B16" s="24" t="n">
-        <v>0</v>
+          <t>P013</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>RESEA RCH ARTICL E AI-Driven sleep staging from actigraphy and heart rate</t>
+        </is>
       </c>
       <c r="C16" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="24" t="n">
-        <v>0</v>
+      <c r="D16" s="54" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
       </c>
       <c r="E16" s="24" t="n">
         <v>0</v>
@@ -9138,17 +9203,21 @@
     <row r="17" ht="50.25" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>G014</t>
-        </is>
-      </c>
-      <c r="B17" s="25" t="n">
-        <v>0</v>
+          <t>P014</t>
+        </is>
+      </c>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>ID: pone.0332577 — 2025/11/1 — page 1 — #1 PLOS ONE OPEN ACCESS</t>
+        </is>
       </c>
       <c r="C17" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="25" t="n">
-        <v>0</v>
+      <c r="D17" s="55" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
       </c>
       <c r="E17" s="25" t="n">
         <v>0</v>
@@ -9184,17 +9253,21 @@
     <row r="18" ht="50.25" customHeight="1">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>G015</t>
-        </is>
-      </c>
-      <c r="B18" s="24" t="n">
-        <v>0</v>
+          <t>P015</t>
+        </is>
+      </c>
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>Review Detection of Sleep Apnea Using Wearable AI: Systematic Review and Meta-Analysis</t>
+        </is>
       </c>
       <c r="C18" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="24" t="n">
-        <v>0</v>
+      <c r="D18" s="54" t="inlineStr">
+        <is>
+          <t>s: Wearable AI shows potential in identifying and classifying sleep apnea, but its current performance is suboptimal for routine clinical use. We recommend concurrent use with traditional assessments until improved evidence supports its reliability. Certified commercial wearables are needed for effectively detecting sleep apnea, predicting its occurrence, and delivering proactive interventions. Researchers should conduct further studies on detecting central sleep apnea, prioritize deep learning...</t>
+        </is>
       </c>
       <c r="E18" s="24" t="n">
         <v>0</v>
@@ -9230,17 +9303,21 @@
     <row r="19" ht="50.25" customHeight="1">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>G016</t>
-        </is>
-      </c>
-      <c r="B19" s="25" t="n">
-        <v>0</v>
+          <t>P016</t>
+        </is>
+      </c>
+      <c r="B19" s="25" t="inlineStr">
+        <is>
+          <t>npj |digital medicine Editorial Published in partnership with Seoul National University Bundang Hospital Challenges and opportunities of deep learning</t>
+        </is>
       </c>
       <c r="C19" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="D19" s="25" t="n">
-        <v>0</v>
+      <c r="D19" s="55" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
       </c>
       <c r="E19" s="25" t="n">
         <v>0</v>
@@ -9276,17 +9353,21 @@
     <row r="20" ht="50.25" customHeight="1">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>G017</t>
-        </is>
-      </c>
-      <c r="B20" s="24" t="n">
-        <v>0</v>
+          <t>P017</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>Citation: Toma, T.I.; Choi, S. An End-to-End Multi-Channel Convolutional Bi-LSTM Network for</t>
+        </is>
       </c>
       <c r="C20" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="D20" s="24" t="n">
-        <v>0</v>
+      <c r="D20" s="54" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
       </c>
       <c r="E20" s="24" t="n">
         <v>0</v>
@@ -9317,6 +9398,91 @@
       </c>
       <c r="N20" s="24" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>P018</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Citation: Alajlan, N.N.; Ibrahim, D.M. DDD TinyML: A TinyML-Based Driver Drowsiness Detection Model</t>
+        </is>
+      </c>
+      <c r="D21" s="56" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>P019</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Academic Editor: Miguel Ángel Carvajal Rodríguez Revised: 3 March 2026</t>
+        </is>
+      </c>
+      <c r="D22" s="56" t="inlineStr">
+        <is>
+          <t>Future work will explore the integration of dry electrodes and multimodal sensors (e.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>P020</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SleepFCN: A Fully Convolutional Deep Learning Framework for Sleep Stage Classiﬁcation Using Single-Channel Electroencephalograms</t>
+        </is>
+      </c>
+      <c r="D23" s="56" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>P021</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Vol.:(0123456789) 1 3 A lightweight automatic sleep staging method for children</t>
+        </is>
+      </c>
+      <c r="D24" s="56" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>P022</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SLEEP, 2025, 48, 1–14 Advance access publication 19 August 2024 Original Article</t>
+        </is>
+      </c>
+      <c r="D25" s="56" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -9348,7 +9514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9487,12 +9653,12 @@
       </c>
       <c r="B4" s="24" t="inlineStr">
         <is>
-          <t>CNN-LSTM Hybrid</t>
-        </is>
-      </c>
-      <c r="C4" s="24" t="inlineStr">
-        <is>
-          <t>Deep Learning</t>
+          <t>DeepSleepNet: a Model for Automatic Sleep Stage Scoring based on Raw Single-Channel EEG Akara Supratak, Hao Dong, Chao Wu, and Yike Guo*</t>
+        </is>
+      </c>
+      <c r="C4" s="54" t="inlineStr">
+        <is>
+          <t>From Abstract: —The present study proposes a deep learning model, named DeepSleepNet, for automatic sleep stage scoring based on raw single-channel EEG. Most of the existing methods rely on hand-engineered features which require prior knowledge of sleep analysis. Only a few of them encode the temporal information such as transition rules, which is important for identifying the next sleep stages, into the extracted features. In the proposed model, we utilize Convolutional Neural Networks to extract time- invari...</t>
         </is>
       </c>
       <c r="D4" s="24" t="inlineStr">
@@ -9566,14 +9732,20 @@
       </c>
     </row>
     <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="B5" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="24" t="n">
-        <v>0</v>
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>arXiv:1809.10932v3  [cs.LG]  2 Feb 2019 SeqSleepNet: End-to-End Hierarchical Recurrent Neural Network for Sequence-to-Sequence</t>
+        </is>
+      </c>
+      <c r="C5" s="54" t="inlineStr">
+        <is>
+          <t>[29], [30] but also modern deep neural networks [9]– [11], [13], [23], [25]. The work in [8] showed that while the contextual input does not always lead to performance improvement regardless of the choice of classiﬁcation mode l, it also suffers from the modelling ambiguity and high com- putational overhead. The one-to-many scheme is orthogonal to the many-to-one scheme and was recently proposed in [8] with the concept of contextual output . Under this scheme, a multitask model receives a singl...</t>
+        </is>
       </c>
       <c r="D5" s="24" t="n">
         <v>0</v>
@@ -9622,14 +9794,20 @@
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="B6" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="25" t="n">
-        <v>0</v>
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>P003</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>Article 1 Automatic sleep staging by a hybrid model based on deep 1D- 2 ResNet-SE and LSTM with single-channel raw EEG signals 3</t>
+        </is>
+      </c>
+      <c r="C6" s="55" t="inlineStr">
+        <is>
+          <t>137...</t>
+        </is>
       </c>
       <c r="D6" s="25" t="n">
         <v>0</v>
@@ -9678,14 +9856,20 @@
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="B7" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="24" t="n">
-        <v>0</v>
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>P004</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>An Attention-Based Deep Learning Approach for Sleep Stage Classiﬁcation With Single-Channel EEG</t>
+        </is>
+      </c>
+      <c r="C7" s="54" t="inlineStr">
+        <is>
+          <t>to classify EEG signals into corresponding sleep stages. These methods usually consist of two steps, namely, manual feature extraction and sl eep stage classiﬁcation. First, they design and extract various features from time and fre- quency domains. Feature selection algorithms are often applied to further select the most discriminative features. Second, the selected features are then f ed into conventional machine learning models for sleep stage classiﬁcation, such as Naive Bayes [8], support...</t>
+        </is>
       </c>
       <c r="D7" s="24" t="n">
         <v>0</v>
@@ -9734,14 +9918,20 @@
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="B8" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="25" t="n">
-        <v>0</v>
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>1 An Unsupervised TinyML Approach with Efficient Edge AI for Effective Stress and Sleep</t>
+        </is>
+      </c>
+      <c r="C8" s="55" t="inlineStr">
+        <is>
+          <t>like signal normalization an d  transformations tailored for the LSM9DS1 sensor  package. UTMESS employs a transfer learning  approach with MobileNetV2 for classifying  physiological data and uses LSTM autoencoders to  detect time-based anomalies. It can run efficiently on  edge devices using TensorFlow Lite and embedded  2025 International Conference on Recent Innovation in Science Engineering and Technology (ICRISET) | 979-8-3315-5833-8/25/$31.00 ©2025 IEEE | DOI: 10.1109/ICRISET64803.2025.11...</t>
+        </is>
       </c>
       <c r="D8" s="25" t="n">
         <v>0</v>
@@ -9790,14 +9980,20 @@
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="B9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="24" t="n">
-        <v>0</v>
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>P006</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Digital Object Identifier 10.1 109/ACCESS.2018.2849822 A Smart System for Sleep Monitoring by Integrating IoT With Big Data Analytics</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>From Abstract: Obtrusive sleep apnea (OSA) is one of the most important sleep disorders because it has a direct adverse impact on the quality of life. Intellectual deterioration, decreased psychomotor performance, behavior, and personality disorders are some of the consequences of OSA. Therefore, a real-time monitoring of this disorder is a critical need in healthcare solutions. There are several systems for OSA detection. Nevertheless, despite their promising results, these systems not guiding their treatmen...</t>
+        </is>
       </c>
       <c r="D9" s="24" t="n">
         <v>0</v>
@@ -9846,14 +10042,20 @@
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="B10" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="25" t="n">
-        <v>0</v>
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>P007</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>Academic Editor: Luca Mesin Revised: 28 October 2025 Published: 31 October 2025</t>
+        </is>
+      </c>
+      <c r="C10" s="55" t="inlineStr">
+        <is>
+          <t>From Abstract: Sleep is a fundamental biological process essential for health and homeostasis. Traditionally investigated through laboratory-based polysomnography (PSG), sleep research has under- gone a paradigm shift with the advent of wearable technologies that enable non-invasive, long-term, and real-world monitoring. This review traces the evolution from early analog and actigraphic methods to current multi-sensor and AI-driven wearable systems. We summarize major technological milestones, including the t...</t>
+        </is>
       </c>
       <c r="D10" s="25" t="n">
         <v>0</v>
@@ -9902,14 +10104,20 @@
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="B11" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="24" t="n">
-        <v>0</v>
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>P008</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>Citation: Srivastava, P .; Shah, N.; Jaiswal, K. Microcontroller-Based EdgeML: Health Monitoring for Stress</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>This section describes the methodology followed in this research, outlining data collection, model development, deployment, and evaluation. The process flow of the entire methodology is depicted in Figure 1. Eng. Proc.2024, 78, 3 3 of 8 Figure 1. Flowchart of the proposed methodology....</t>
+        </is>
       </c>
       <c r="D11" s="24" t="n">
         <v>0</v>
@@ -9958,14 +10166,20 @@
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="B12" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="25" t="n">
-        <v>0</v>
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>P009</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>Federated Learning for Sleep Stage Classification on Edge Devices via a Model-Agnostic Meta-Learning-Based Pre-Trained Model</t>
+        </is>
+      </c>
+      <c r="C12" s="55" t="inlineStr">
+        <is>
+          <t>for monitoring sleep quality and stages [6]. At  present, polysomnography (PSG) is considered the gold  standard technique for assessing sleep quality and states  following the technical specifications outlined by the  American Academy of Sleep Medicine (AASM) [7]. During  a designated sleep time, sleep specialists use PSG to record  various physiological signals such as electroencephalogram  (EEG), electrocardiogram (ECG), electrooculogram (EOG),  and electromyography (EMG). Sleep specialists...</t>
+        </is>
       </c>
       <c r="D12" s="25" t="n">
         <v>0</v>
@@ -10014,14 +10228,20 @@
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="B13" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="24" t="n">
-        <v>0</v>
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>P010</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>Validation of an automated wireless system to monitor sleep in healthy adults JOHN R. SHAMBROOM 1 , STEPHAN E. FA ´ BREGAS 1 and JACK JOHNSTONE 2</t>
+        </is>
+      </c>
+      <c r="C13" s="54" t="inlineStr">
+        <is>
+          <t>Subjects Twenty-nine subjects were enrolled and completed the protocol. However, three consecutive sleep recordings were lost due to a technician error. Of the 26 remaining subjects, 50% were female and the average age [± standard deviation (SD)] was 38 (± 13) years, ranging from 19 to 60 years. Inclusion criteria were as follows: healthy adults (18– 65 years), with no physical or mental health complaints, with a body mass index between 18.6 and 30.0, and a willingness to abstain from alcohol,...</t>
+        </is>
       </c>
       <c r="D13" s="24" t="n">
         <v>0</v>
@@ -10070,14 +10290,20 @@
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="B14" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="25" t="n">
-        <v>0</v>
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>P011</t>
+        </is>
+      </c>
+      <c r="B14" s="25" t="inlineStr">
+        <is>
+          <t>Review Wearable Artificial Intelligence for Sleep Disorders: Scoping Review</t>
+        </is>
+      </c>
+      <c r="C14" s="55" t="inlineStr">
+        <is>
+          <t>: Seven electronic databases (MEDLINE, PsycINFO, Embase, IEEE Xplore, ACM Digital Library, Google Scholar, and Scopus) were searched for peer-reviewed literature published before March 2024. Keywords were selected based on 3 domains: sleep disorders, AI, and wearable devices. The primary selection criterion was the inclusion of studies that utilized AI algorithms to detect or predict various sleep disorders using data from wearable devices. Study selection was conducted in 2 steps: first, by rev...</t>
+        </is>
       </c>
       <c r="D14" s="25" t="n">
         <v>0</v>
@@ -10126,14 +10352,20 @@
       </c>
     </row>
     <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="B15" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="24" t="n">
-        <v>0</v>
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>P012</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>RESEA RCH ARTICL E Multi-scale ResNet and BiGRU automatic sleep staging based on attention mechanism</t>
+        </is>
+      </c>
+      <c r="C15" s="54" t="inlineStr">
+        <is>
+          <t>From Abstract: Sleep staging is the basis of sleep evaluation and a key step in the diagnosis of sleep- related diseases. Despite being useful, the existing sleep staging methods have several dis- advantages, such as relying on artificial feature extraction, failing to recognize temporal sequence patterns in the long-term associated data, and reaching the accuracy upper limit of sleep staging. Hence, this paper proposes an automatic Electroencephalo gram (EEG) sleep signal staging model, which based on Multi-...</t>
+        </is>
       </c>
       <c r="D15" s="24" t="n">
         <v>0</v>
@@ -10182,14 +10414,20 @@
       </c>
     </row>
     <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="B16" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="25" t="n">
-        <v>0</v>
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t>P013</t>
+        </is>
+      </c>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>RESEA RCH ARTICL E AI-Driven sleep staging from actigraphy and heart rate</t>
+        </is>
+      </c>
+      <c r="C16" s="55" t="inlineStr">
+        <is>
+          <t>From Abstract: Sleep is an important indicator of a person’s health, and its accurate and cost-effective quantification is of great value in healthcare. The gold standard for sleep assessment and the clinical diagnosis of sleep disorders is polysomnogra phy (PSG). However, PSG requires an overnight clinic visit and trained technicians to score the obtained multimodality data. Wrist-worn consumer devices, such as smartwatches, are a promising alternative to PSG because of their small form factor, continuous mo...</t>
+        </is>
       </c>
       <c r="D16" s="25" t="n">
         <v>0</v>
@@ -10238,14 +10476,20 @@
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="B17" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="24" t="n">
-        <v>0</v>
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>P014</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>ID: pone.0332577 — 2025/11/1 — page 1 — #1 PLOS ONE OPEN ACCESS</t>
+        </is>
+      </c>
+      <c r="C17" s="54" t="inlineStr">
+        <is>
+          <t>From Abstract: Driver drowsiness is a leading cause of traffic accidents and fatalities, highlighting the urgent need for intelligent systems capable of real-time fatigue detection. Although recent advancements in machine learning (ML) and deep learning (DL) have signifi- cantly improved detection accuracy, most existing models are computationally demand- ing and not well-suited for deployment in resource-limited environments such as micro- controllers. While the emerging domain of TinyML presents promising a...</t>
+        </is>
       </c>
       <c r="D17" s="24" t="n">
         <v>0</v>
@@ -10294,14 +10538,20 @@
       </c>
     </row>
     <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="B18" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" s="25" t="n">
-        <v>0</v>
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>P015</t>
+        </is>
+      </c>
+      <c r="B18" s="25" t="inlineStr">
+        <is>
+          <t>Review Detection of Sleep Apnea Using Wearable AI: Systematic Review and Meta-Analysis</t>
+        </is>
+      </c>
+      <c r="C18" s="55" t="inlineStr">
+        <is>
+          <t>: Our search was conducted in 6 electronic databases. This review included English research articles evaluating wearable AI’s performance in identifying sleep apnea, distinguishing its type, and gauging its severity. Two researchers independently conducted study selection, extracted data, and assessed the risk of bias using an adapted Quality Assessment of Studies of Diagnostic Accuracy-Revised tool. We used both narrative and statistical techniques for evidence synthesis. Results: Among 615 stu...</t>
+        </is>
       </c>
       <c r="D18" s="25" t="n">
         <v>0</v>
@@ -10350,14 +10600,20 @@
       </c>
     </row>
     <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="B19" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="24" t="n">
-        <v>0</v>
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>P016</t>
+        </is>
+      </c>
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>npj |digital medicine Editorial Published in partnership with Seoul National University Bundang Hospital Challenges and opportunities of deep learning</t>
+        </is>
+      </c>
+      <c r="C19" s="54" t="inlineStr">
+        <is>
+          <t>Not extracted</t>
+        </is>
       </c>
       <c r="D19" s="24" t="n">
         <v>0</v>
@@ -10403,6 +10659,108 @@
       </c>
       <c r="R19" s="24" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>P017</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Citation: Toma, T.I.; Choi, S. An End-to-End Multi-Channel Convolutional Bi-LSTM Network for</t>
+        </is>
+      </c>
+      <c r="C20" s="56" t="inlineStr">
+        <is>
+          <t>From Abstract: : Sleep stage detection from polysomnography (PSG) recordings is a widely used method of monitoring sleep quality. Despite signiﬁcant progress in the development of machine-learning (ML)-based and deep-learning (DL)-based automatic sleep stage detection schemes focusing on single-channel PSG data, such as single-channel electroencephalogram (EEG), electrooculogram (EOG), and electromyogram (EMG), developing a standard model is still an active subject of research. Often, the use of a single sourc...</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>P018</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Citation: Alajlan, N.N.; Ibrahim, D.M. DDD TinyML: A TinyML-Based Driver Drowsiness Detection Model</t>
+        </is>
+      </c>
+      <c r="C21" s="56" t="inlineStr">
+        <is>
+          <t>From Abstract: : Driver drowsiness is one of the main causes of trafﬁc accidents today. In recent years, driver drowsiness detection has suffered from issues integrating deep learning (DL) with Internet-of- things (IoT) devices due to the limited resources of IoT devices, which pose a challenge to fulﬁlling DL models that demand large storage and computation. Thus, there are challenges to meeting the requirements of real-time driver drowsiness detection applications that need short latency and lightweight comp...</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>P019</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Academic Editor: Miguel Ángel Carvajal Rodríguez Revised: 3 March 2026</t>
+        </is>
+      </c>
+      <c r="C22" s="56" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>P020</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SleepFCN: A Fully Convolutional Deep Learning Framework for Sleep Stage Classiﬁcation Using Single-Channel Electroencephalograms</t>
+        </is>
+      </c>
+      <c r="C23" s="56" t="inlineStr">
+        <is>
+          <t>using RNNs or even attention mechanisms. Moreover, the SleepFCN exhibits more generality for the breath-related distortions in individuals’ sleep. Furthermore, avoiding fully connected layers provides the model ﬂexibility to varying dimensions. It is beneﬁcial for sleep technicians to have a relatively accurate and fast model to train and test over unseen data. Therefore, the motives for future research in the ﬁeld of sleep stage classiﬁcation can be pruning the model to reduce the parameters f...</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>P021</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Vol.:(0123456789) 1 3 A lightweight automatic sleep staging method for children</t>
+        </is>
+      </c>
+      <c r="C24" s="56" t="inlineStr">
+        <is>
+          <t>From Abstract: With the development of telemedicine and edge computing, edge artificial intelligence (AI)  will become a new development trend for smart medicine. On the other hand, nearly one- third of children suffer from sleep disorders. However, all existing sleep staging methods  are for adults. Therefore, we adapted edge AI to develop a lightweight automatic sleep  staging method for children using single-channel EEG. The trained sleep staging model  will be deployed to edge smart devices so that the sl...</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>P022</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SLEEP, 2025, 48, 1–14 Advance access publication 19 August 2024 Original Article</t>
+        </is>
+      </c>
+      <c r="C25" s="56" t="inlineStr">
+        <is>
+          <t>From Abstract: The ability to assess sleep at home, capture sleep stages, and detect the occurrence of apnea (without on-body sensors) simply by  analyzing the radio waves bouncing off people’s bodies while they sleep is quite powerful. Such a capability would allow for longi - tudinal data collection in patients’ homes, informing our understanding of sleep and its interaction with various diseases and their  therapeutic responses, both in clinical trials and routine care. In this article, we develop an adva...</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>